<commit_message>
Add complexity tiers and work plan to FXR90 review fix list
Adds a Work Plan sheet ordering all 36 review issues by complexity, plus
Complexity and Blocked-on columns on the Fix List sheet.

- Simple (15): self-contained edits, no unknowns
- Medium (10): mechanical but wide-reaching, or need one fact confirmed
- Complex (7): schema design work, or scope not yet bounded

Effort concentrates in Operating Mode (#27-#31). Eight items are blocked
on Mayur or dev input rather than on doc work.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RestAPI/developer_feedback/FXR90_fix_list.xlsx
+++ b/RestAPI/developer_feedback/FXR90_fix_list.xlsx
@@ -10,10 +10,12 @@
     <sheet name="0. Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="1. Fix List" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="2. To Verify" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="3. Work Plan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Fix List'!$A$3:$M$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Fix List'!$A$3:$O$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. To Verify'!$A$3:$F$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. Work Plan'!$A$3:$E$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -58,7 +60,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +107,21 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -132,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,6 +188,18 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -538,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -832,10 +861,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr"/>
-    </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
@@ -901,6 +927,90 @@
       <c r="B37" s="3" t="inlineStr">
         <is>
           <t>#4, #7, #14 - schema/examples only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>COMPLEXITY BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>15 items - self-contained edits, no unknowns. Includes #2, the highest-impact item on the list. Roughly half the list can be done today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>10 items - mechanical but touch many places, or need one fact confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>7 items (11 counting the merged ones) - real schema design work, or scope you cannot bound yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Where the effort actually is</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Operating Mode (#27, #28, #29, #31) = getMode.md + setMode.md + the mode schemas. That is MOST of the real work. Everything else is small by comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED - SEND THIS TO MAYUR FIRST</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>8 items are blocked on others, not on you</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>#3 (what verbose excludes)  #8 (the payload)  #9 (expandAll)  #12 (MQTTGC name)  #15 (log levels)  #17 (which server)  #23 (powerNegotiation spelling)  #31 (dock door / ATR). Also #16 (strip the model enum?) and #22/#26 need dev input. Send these BEFORE starting, or you will finish the easy 15 and stall.</t>
         </is>
       </c>
     </row>
@@ -915,7 +1025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -931,6 +1041,8 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -940,7 +1052,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="32" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -1005,6 +1116,16 @@
       <c r="M3" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="N3" s="6" t="inlineStr">
+        <is>
+          <t>Complexity</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr">
+        <is>
+          <t>Blocked on</t>
         </is>
       </c>
     </row>
@@ -1068,6 +1189,12 @@
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr"/>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="n">
@@ -1129,6 +1256,12 @@
         </is>
       </c>
       <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
@@ -1190,6 +1323,16 @@
         </is>
       </c>
       <c r="M6" s="7" t="inlineStr"/>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O6" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - what does verbose:true exclude?</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
@@ -1251,6 +1394,12 @@
         </is>
       </c>
       <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
@@ -1312,6 +1461,12 @@
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr"/>
+      <c r="N8" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
@@ -1373,6 +1528,12 @@
         </is>
       </c>
       <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
@@ -1434,6 +1595,12 @@
         </is>
       </c>
       <c r="M10" s="7" t="inlineStr"/>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
@@ -1495,6 +1662,16 @@
         </is>
       </c>
       <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O11" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - the correct WebSocket payload</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
@@ -1556,6 +1733,16 @@
         </is>
       </c>
       <c r="M12" s="7" t="inlineStr"/>
+      <c r="N12" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O12" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - what is 'expandAll'?</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n">
@@ -1617,6 +1804,12 @@
         </is>
       </c>
       <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
@@ -1678,6 +1871,12 @@
         </is>
       </c>
       <c r="M14" s="7" t="inlineStr"/>
+      <c r="N14" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n">
@@ -1739,6 +1938,16 @@
         </is>
       </c>
       <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O15" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - exact name of 'keyboard' / 'MQTTGC'</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
@@ -1800,6 +2009,12 @@
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr"/>
+      <c r="N16" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n">
@@ -1861,6 +2076,12 @@
         </is>
       </c>
       <c r="M17" s="7" t="inlineStr"/>
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
@@ -1922,6 +2143,16 @@
         </is>
       </c>
       <c r="M18" s="7" t="inlineStr"/>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O18" s="18" t="inlineStr">
+        <is>
+          <t>DEV - which log levels are real?</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n">
@@ -1983,6 +2214,16 @@
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr"/>
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O19" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - strip the other 4 models or keep?</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
@@ -2044,6 +2285,16 @@
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr"/>
+      <c r="N20" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O20" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - which 'server'? NTP or cloud endpoint?</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="n">
@@ -2105,6 +2356,12 @@
         </is>
       </c>
       <c r="M21" s="7" t="inlineStr"/>
+      <c r="N21" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
@@ -2166,6 +2423,12 @@
         </is>
       </c>
       <c r="M22" s="7" t="inlineStr"/>
+      <c r="N22" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="n">
@@ -2227,6 +2490,12 @@
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr"/>
+      <c r="N23" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
@@ -2288,6 +2557,12 @@
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr"/>
+      <c r="N24" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O24" s="7" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="7" t="n">
@@ -2349,6 +2624,16 @@
         </is>
       </c>
       <c r="M25" s="7" t="inlineStr"/>
+      <c r="N25" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O25" s="18" t="inlineStr">
+        <is>
+          <t>DEV - correct powerSource values</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
@@ -2410,6 +2695,16 @@
         </is>
       </c>
       <c r="M26" s="7" t="inlineStr"/>
+      <c r="N26" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O26" s="18" t="inlineStr">
+        <is>
+          <t>DEV - exact powerNegotiation enum spelling</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="n">
@@ -2471,6 +2766,12 @@
         </is>
       </c>
       <c r="M27" s="7" t="inlineStr"/>
+      <c r="N27" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
@@ -2532,6 +2833,12 @@
         </is>
       </c>
       <c r="M28" s="7" t="inlineStr"/>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="n">
@@ -2593,6 +2900,16 @@
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr"/>
+      <c r="N29" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O29" s="18" t="inlineStr">
+        <is>
+          <t>DEV - exact readerLocation name + lat/long structure</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
@@ -2654,6 +2971,12 @@
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr"/>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O30" s="7" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="7" t="n">
@@ -2715,6 +3038,12 @@
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr"/>
+      <c r="N31" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
@@ -2776,6 +3105,12 @@
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr"/>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O32" s="7" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="n">
@@ -2837,6 +3172,12 @@
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr"/>
+      <c r="N33" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
@@ -2898,6 +3239,16 @@
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr"/>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O34" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - is 'dock door' ATR-only?</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="n">
@@ -2959,6 +3310,12 @@
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr"/>
+      <c r="N35" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="n">
@@ -3020,6 +3377,12 @@
         </is>
       </c>
       <c r="M36" s="7" t="inlineStr"/>
+      <c r="N36" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="n">
@@ -3081,6 +3444,12 @@
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr"/>
+      <c r="N37" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="n">
@@ -3142,6 +3511,12 @@
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr"/>
+      <c r="N38" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="n">
@@ -3203,9 +3578,15 @@
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr"/>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:M39"/>
+  <autoFilter ref="A3:O39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3530,4 +3911,803 @@
   <autoFilter ref="A3:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="88" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>WORK PLAN BY COMPLEXITY - do them in this order</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Why it is this tier</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Blocked on</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>App LED: remove blue</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Delete 'blue' from SetAppledRequest.color.enum. One word. KEEP blue in SetStackledRequest.</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Get/Set Mode example: Gen2X -&gt; Gen2</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Three examples say GEN2X. Find and replace. HIGHEST CUSTOMER IMPACT ON THE LIST - this is the one that generates SPRs.</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>inventoryProtocol enum</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>ALREADY DONE - enum is already [GEN2X, GEN2, HYBRID]. Verify and close.</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>16</v>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Model enum</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>FXR90 is ALREADY present. Only decision: strip the other 4 models or keep them.</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>32</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Remove XML</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>GetConfigResponse.xml and SetConfigMqttRequest.xml - delete two properties.</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Delete stray mode fields</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>PART A ONLY: delete component, payload, linkProfile from SetModeRequest. Part B (beams / dock door) is Complex - see below.</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Password description</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Mayur gave the exact replacement sentence at 00:19:08. Paste it.</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Password examples</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Add an rfid-adm example beside the existing admin one.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>doNotPersist: remove BLE</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Remove BLE from the description and the persistence table.</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Control-mode note</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Add one sentence: Get Start/Stop IS supported in control mode.</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>getVersion empty fields</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Add 'currently always returns empty' to two field descriptions.</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>11+20</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Remove Stack LED</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Delete the /cloud/stack-led path and its 3 components. One fix closes two issues.</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Do-not-duplicate guardrail</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>NO EDIT AT ALL. This is a warning for items 27-31.</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Fix broken links</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Simple IF the count is small. Audit first.</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Simple</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>17</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Server-delete limitation</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>One sentence - once you know which 'server' is meant.</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>12+34</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Remove GCP + keyboard-emulation</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Strings are scattered across EVERY connection-type description in the file. Tedious, not hard. Do both together.</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR - exact name of MQTTGC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>WebSocket: remove unsupported fields</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>Remove verifyHost / verifyPeer. Blocked only on what 'expandAll' actually is.</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>WebSocket payload</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Easy once Mayur sends the payload he referenced in the comment.</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>BLE version notes</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>Touches 4 .md files. Mechanical.</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Split uap0 / mlan0 examples</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Separate the examples and add the mutual-exclusion note.</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>33</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Add AWS + Azure connectors</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>Update the connector list and capabilities.endpointTypesSupported.</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>powerSource: DC -&gt; Power Brick</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>powerSource has NO enum today. Adding one is easy - you need the correct values.</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>powerNegotiation values</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>powerNegotiation has NO enum today. Same as above.</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>DEV - exact spelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>15</v>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Log levels</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Trivial edit. Blocked on which of off / fatal / trace / extra are real.</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>tagMetaData: add readerLocation</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Add READER_LOCATION to the enum - need the exact name and lat/long structure.</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>27+28+29</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>OPERATING MODE - THE BIG ONE</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>modeSpecificSettings, selects, accesses, radioStartConditions, radioStopConditions, rssiFilter, readerLocation are ALL absent from properties - several exist only inside examples. Deeply nested objects to author from scratch, on BOTH Get and Set. Plus keep antennaStopCondition distinct from radioStopConditions. Treat as one project, not three tickets. THIS IS MOST OF THE REAL EFFORT.</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>36</v>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Config schema completeness</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>'Include every supported parameter, remove every unsupported one' - unbounded until someone defines the supported set. Swallows 32, 33, 34.</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Network schema completeness</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Same shape as 36, for the network schema.</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>verbose flag</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Does not exist in the spec AND nobody knows what verbose:true excludes. HARD BLOCKED.</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>35</v>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Error-code schema</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>New schema. error_codes.json exists at repo root but is not wired in.</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="C34" s="7" t="inlineStr">
+        <is>
+          <t>Docs / schema sync</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>The umbrella item - effectively 'do all the others'.</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Replace stale examples</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Scope unknown until every example block is audited.</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>Complex</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>31</v>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
+          <t>Remove beams / directionality / dock door</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>PART B: removing beams and directionality is easy. Confirming dock door / ATR is not, and it is unresolved.</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>MAYUR</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:E36"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>